<commit_message>
data: MI355X MXFP4 EP=8 TP=8 profiling (chat c=4)
</commit_message>
<xml_diff>
--- a/results/mi355x_dsr_mxfp4/mi355x_dsr_mxfp4_mtp0_ep8_tp8_rocm711_profiling/prefill_breakdown.xlsx
+++ b/results/mi355x_dsr_mxfp4/mi355x_dsr_mxfp4_mtp0_ep8_tp8_rocm711_profiling/prefill_breakdown.xlsx
@@ -471,22 +471,22 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>189.08</v>
+        <v>217.2</v>
       </c>
       <c r="D2" t="n">
-        <v>69.90000000000001</v>
+        <v>72.2</v>
       </c>
       <c r="E2" t="n">
-        <v>201.239</v>
+        <v>230.799</v>
       </c>
       <c r="F2" t="n">
-        <v>74.40000000000001</v>
+        <v>76.8</v>
       </c>
       <c r="G2" t="n">
-        <v>252.7139024390244</v>
+        <v>246.8280975609756</v>
       </c>
       <c r="H2" t="n">
-        <v>265.1149756097561</v>
+        <v>259.5695853658536</v>
       </c>
     </row>
     <row r="3">
@@ -496,13 +496,13 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>12.159</v>
+        <v>13.599</v>
       </c>
       <c r="D3" t="n">
         <v>4.5</v>
       </c>
       <c r="G3" t="n">
-        <v>12.40107317073171</v>
+        <v>12.74148780487805</v>
       </c>
     </row>
     <row r="4">
@@ -517,22 +517,22 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>64.72</v>
+        <v>65.28</v>
       </c>
       <c r="D4" t="n">
-        <v>23.9</v>
+        <v>21.7</v>
       </c>
       <c r="E4" t="n">
-        <v>64.72</v>
+        <v>65.28</v>
       </c>
       <c r="F4" t="n">
-        <v>23.9</v>
+        <v>21.7</v>
       </c>
       <c r="G4" t="n">
-        <v>64.5730731707317</v>
+        <v>64.6990487804878</v>
       </c>
       <c r="H4" t="n">
-        <v>64.5730731707317</v>
+        <v>64.6990487804878</v>
       </c>
     </row>
     <row r="5">
@@ -547,22 +547,22 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>4.639</v>
+        <v>4.599</v>
       </c>
       <c r="D5" t="n">
-        <v>1.7</v>
+        <v>1.5</v>
       </c>
       <c r="E5" t="n">
-        <v>4.639</v>
+        <v>4.599</v>
       </c>
       <c r="F5" t="n">
-        <v>1.7</v>
+        <v>1.5</v>
       </c>
       <c r="G5" t="n">
-        <v>4.731756097560976</v>
+        <v>4.6</v>
       </c>
       <c r="H5" t="n">
-        <v>4.731756097560976</v>
+        <v>4.6</v>
       </c>
     </row>
     <row r="6">
@@ -573,7 +573,7 @@
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="n">
-        <v>270.598</v>
+        <v>300.678</v>
       </c>
       <c r="D6" t="n">
         <v>100</v>
@@ -583,7 +583,7 @@
         <v>100</v>
       </c>
       <c r="G6" t="n">
-        <v>334.4198048780488</v>
+        <v>328.8686341463414</v>
       </c>
       <c r="H6" t="inlineStr"/>
     </row>
@@ -644,13 +644,13 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>189.08</v>
+        <v>217.2</v>
       </c>
       <c r="D2" t="n">
-        <v>189.08</v>
+        <v>217.2</v>
       </c>
       <c r="E2" t="n">
-        <v>69.90000000000001</v>
+        <v>72.2</v>
       </c>
     </row>
     <row r="3">
@@ -663,13 +663,13 @@
         <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>64.72</v>
+        <v>65.28</v>
       </c>
       <c r="D3" t="n">
-        <v>64.72</v>
+        <v>65.28</v>
       </c>
       <c r="E3" t="n">
-        <v>23.9</v>
+        <v>21.7</v>
       </c>
     </row>
     <row r="4">
@@ -682,10 +682,10 @@
         <v>1</v>
       </c>
       <c r="C4" t="n">
-        <v>12.159</v>
+        <v>13.599</v>
       </c>
       <c r="D4" t="n">
-        <v>12.159</v>
+        <v>13.599</v>
       </c>
       <c r="E4" t="n">
         <v>4.5</v>
@@ -701,13 +701,13 @@
         <v>1</v>
       </c>
       <c r="C5" t="n">
-        <v>4.639</v>
+        <v>4.599</v>
       </c>
       <c r="D5" t="n">
-        <v>4.639</v>
+        <v>4.599</v>
       </c>
       <c r="E5" t="n">
-        <v>1.7</v>
+        <v>1.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>